<commit_message>
Case-study editor: record a case study on its IFC model
A static web page (docs/source/_extra/editor) that reads and draws the IFC
model with IFC-Lite, edits the case study in forms generated from the
workbook's sheets, assigns walls to facades by selecting them in 3D, and
saves the case study into the IFC file: the whole record on the
IfcProject (HSV_CaseRecord), facade, unit, masonry type and
vulnerabilities on each element (HSV_Facade), MQI categories on each
masonry material (HMO_MasonryQuality).

python -m core.knowledge_graph build/convert now read a case study from
the saved IFC file, a case.json or a workbook; facade elements become
parts of their facade in the graph. SERA-AIMS recorded in
aggregate_1_case.ifc with its walls assigned. Version 1.1.0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/source/_extra/case_template.xlsx
+++ b/docs/source/_extra/case_template.xlsx
@@ -670,6 +670,11 @@
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <t>Name of its masonry type (MasonryTypes)</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>GlobalIds of its IFC elements, separated by ; (set by the editor)</t>
       </text>
     </comment>
   </commentList>
@@ -2120,13 +2125,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2148,6 +2154,11 @@
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>masonry_type</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>elements</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Editor and docs: the user records morphological characteristics, not MQI parameters
The seven values entered for each masonry type are categories of morphological
characteristics; the scores of the quality index are assigned by the reasoner.
The labels of the editor, the help text of the schema and workbooks, the case-
study and workflow pages and the two editor figures now say so. Field names and
the file format are unchanged, so existing records still load.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/source/_extra/case_template.xlsx
+++ b/docs/source/_extra/case_template.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Project" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Organisations" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="People" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Activities" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Documents" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Units" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Facades" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Photos" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Connections" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Openings" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Vulnerabilities" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="MasonryTypes" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Measured" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="_lists" sheetId="14" state="hidden" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Organisations" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activities" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Units" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Facades" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connections" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Openings" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vulnerabilities" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MasonryTypes" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measured" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_lists" sheetId="14" state="hidden" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -294,37 +294,37 @@
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>MQI category: unit dimensions</t>
+        <t>Morphological characteristic: unit dimensions</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>MQI category: unit shape</t>
+        <t>Morphological characteristic: unit shape</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>MQI category: unit material</t>
+        <t>Morphological characteristic: unit material</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>MQI category: mortar quality</t>
+        <t>Morphological characteristic: mortar quality</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>MQI category: horizontal joints</t>
+        <t>Morphological characteristic: horizontal joints</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
-        <t>MQI category: vertical joints</t>
+        <t>Morphological characteristic: vertical joints</t>
       </text>
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>MQI category: wall connections</t>
+        <t>Morphological characteristic: wall connections</t>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
@@ -394,12 +394,12 @@
     </comment>
     <comment ref="W1" authorId="0" shapeId="0">
       <text>
-        <t>Lower variant, as parameter=value; ... (optional)</t>
+        <t>Lower variant, as characteristic=category; ... (optional)</t>
       </text>
     </comment>
     <comment ref="X1" authorId="0" shapeId="0">
       <text>
-        <t>Upper variant, as parameter=value; ... (optional)</t>
+        <t>Upper variant, as characteristic=category; ... (optional)</t>
       </text>
     </comment>
   </commentList>
@@ -1239,7 +1239,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B500" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
       <formula1>=_lists!$L$2:$L$9</formula1>
     </dataValidation>
   </dataValidations>
@@ -1407,25 +1407,25 @@
     </row>
   </sheetData>
   <dataValidations count="7">
-    <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C2:C500" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
       <formula1>=_lists!$A$2:$A$4</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D500" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
       <formula1>=_lists!$B$2:$B$5</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E500" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
       <formula1>=_lists!$C$2:$C$9</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F500" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
       <formula1>=_lists!$D$2:$D$5</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G500" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
       <formula1>=_lists!$E$2:$E$4</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H500" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
       <formula1>=_lists!$F$2:$F$4</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I500" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
       <formula1>=_lists!$G$2:$G$4</formula1>
     </dataValidation>
   </dataValidations>
@@ -2047,7 +2047,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B500" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
       <formula1>=_lists!$H$2:$H$7</formula1>
     </dataValidation>
   </dataValidations>
@@ -2107,10 +2107,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C2:C500" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
       <formula1>=_lists!$I$2:$I$4</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E500" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
       <formula1>=_lists!$K$2:$K$3</formula1>
     </dataValidation>
   </dataValidations>
@@ -2286,7 +2286,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B500" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
       <formula1>=_lists!$J$2:$J$4</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>